<commit_message>
- fixed enable error of RS-422 drivers - gerber files were NOT updated
</commit_message>
<xml_diff>
--- a/01_Altium_Project/BOMs/PowerTower_AdapterUltrazohm_Mouser.xlsx
+++ b/01_Altium_Project/BOMs/PowerTower_AdapterUltrazohm_Mouser.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilflingti66489\Documents\powertower_adapter_uz\01_Altium_Project\BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D2950E-F6EC-46E6-873D-F9EC99E1F23D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12BD53FD-32C1-4F22-AC88-02058D2A04A7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part List Report" sheetId="3" r:id="rId1"/>
     <sheet name="Project Information" sheetId="4" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Part List Report'!$D$9:$M$22</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="140">
   <si>
     <t>Project Full Path</t>
   </si>
@@ -147,9 +150,6 @@
     <t>C14</t>
   </si>
   <si>
-    <t>D2, D3</t>
-  </si>
-  <si>
     <t>F1, F2</t>
   </si>
   <si>
@@ -207,9 +207,6 @@
     <t>C0805C104J5RECTU</t>
   </si>
   <si>
-    <t>150060GS84000, 150060RS86000</t>
-  </si>
-  <si>
     <t>0154001.DR</t>
   </si>
   <si>
@@ -264,9 +261,6 @@
     <t>Capacitor 0805, 50 VDC, 0.1 µF, X7R</t>
   </si>
   <si>
-    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Green, WL-SMCW SMD Mono-color Chip LED Waterclear Red</t>
-  </si>
-  <si>
     <t>Duse OMNI BLOK 154</t>
   </si>
   <si>
@@ -345,9 +339,6 @@
     <t>80-C0805C104J5RECTU</t>
   </si>
   <si>
-    <t>710-150060GS84000, 710-150060RS86000</t>
-  </si>
-  <si>
     <t>576-0154001.DR</t>
   </si>
   <si>
@@ -411,9 +402,6 @@
     <t>EEE-FK0J101V</t>
   </si>
   <si>
-    <t xml:space="preserve">667-EEE-FK0J101V </t>
-  </si>
-  <si>
     <t>Vishay</t>
   </si>
   <si>
@@ -436,6 +424,36 @@
   </si>
   <si>
     <t xml:space="preserve">926-DS26C31TMX/NOPB </t>
+  </si>
+  <si>
+    <t>667-EEE-FK0J101P, ERSATZ: 667-EEE-FK0J101V</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>150060RS86000</t>
+  </si>
+  <si>
+    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Red</t>
+  </si>
+  <si>
+    <t>710-150060RS86000</t>
+  </si>
+  <si>
+    <t>710-150060GS84000</t>
+  </si>
+  <si>
+    <t>WL-SMCW SMD Mono-color Chip LED Waterclear Green</t>
+  </si>
+  <si>
+    <t>150060GS84000</t>
+  </si>
+  <si>
+    <t>D2</t>
   </si>
 </sst>
 </file>
@@ -1299,9 +1317,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>783821</xdr:colOff>
+      <xdr:colOff>791441</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:rowOff>68580</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1691,28 +1709,28 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="5.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="3.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="5.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="23.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="4" customWidth="1"/>
     <col min="7" max="7" width="20" style="4" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="43.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="33.85546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="37.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="43.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="33.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="37.33203125" style="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="37"/>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -1729,7 +1747,7 @@
       <c r="N1" s="41"/>
       <c r="O1" s="17"/>
     </row>
-    <row r="2" spans="1:15" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="38"/>
       <c r="B2" s="29"/>
       <c r="C2" s="29" t="s">
@@ -1748,7 +1766,7 @@
       <c r="M2" s="42"/>
       <c r="N2" s="43"/>
     </row>
-    <row r="3" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="38"/>
       <c r="B3" s="18"/>
       <c r="C3" s="18" t="s">
@@ -1766,7 +1784,7 @@
       <c r="M3" s="18"/>
       <c r="N3" s="21"/>
     </row>
-    <row r="4" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="38"/>
       <c r="B4" s="18"/>
       <c r="C4" s="18" t="s">
@@ -1784,7 +1802,7 @@
       <c r="M4" s="20"/>
       <c r="N4" s="21"/>
     </row>
-    <row r="5" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38"/>
       <c r="B5" s="18"/>
       <c r="C5" s="18" t="s">
@@ -1802,7 +1820,7 @@
       <c r="M5" s="20"/>
       <c r="N5" s="21"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="38"/>
       <c r="B6" s="25"/>
       <c r="C6" s="25"/>
@@ -1818,7 +1836,7 @@
       <c r="M6" s="20"/>
       <c r="N6" s="27"/>
     </row>
-    <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="38"/>
       <c r="B7" s="28"/>
       <c r="C7" s="28" t="s">
@@ -1840,7 +1858,7 @@
       <c r="M7" s="28"/>
       <c r="N7" s="21"/>
     </row>
-    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="38"/>
       <c r="B8" s="24"/>
       <c r="C8" s="24" t="s">
@@ -1850,11 +1868,11 @@
       <c r="F8" s="24"/>
       <c r="G8" s="48">
         <f ca="1">TODAY()</f>
-        <v>44349</v>
+        <v>44369</v>
       </c>
       <c r="H8" s="47">
         <f ca="1">NOW()</f>
-        <v>44349.448239467594</v>
+        <v>44369.425743749998</v>
       </c>
       <c r="I8" s="28"/>
       <c r="J8" s="28"/>
@@ -1863,7 +1881,7 @@
       <c r="M8" s="28"/>
       <c r="N8" s="21"/>
     </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="38"/>
       <c r="B9" s="44" t="s">
         <v>20</v>
@@ -1875,40 +1893,40 @@
         <v>33</v>
       </c>
       <c r="E9" s="45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F9" s="45" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G9" s="45" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H9" s="45" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="K9" s="45" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L9" s="45" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="M9" s="45" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="N9" s="46" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="38"/>
       <c r="B10" s="49">
-        <f t="shared" ref="B10:B21" si="0">ROW(B10) - ROW($B$9)</f>
+        <f t="shared" ref="B10:B22" si="0">ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="61">
@@ -1918,31 +1936,31 @@
         <v>34</v>
       </c>
       <c r="E10" s="56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F10" s="56" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G10" s="57" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H10" s="57" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I10" s="57" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J10" s="77" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K10" s="77" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="L10" s="58"/>
       <c r="M10" s="58"/>
       <c r="N10" s="79"/>
     </row>
-    <row r="11" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="38"/>
       <c r="B11" s="49">
         <f t="shared" si="0"/>
@@ -1955,31 +1973,31 @@
         <v>35</v>
       </c>
       <c r="E11" s="56" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F11" s="56" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G11" s="57" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H11" s="57" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I11" s="57" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J11" s="77" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K11" s="77" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L11" s="58"/>
       <c r="M11" s="58"/>
       <c r="N11" s="79"/>
     </row>
-    <row r="12" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="38"/>
       <c r="B12" s="50">
         <f t="shared" si="0"/>
@@ -1992,31 +2010,31 @@
         <v>36</v>
       </c>
       <c r="E12" s="59" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F12" s="59" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G12" s="59" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H12" s="59" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I12" s="59" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J12" s="78" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K12" s="78" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="L12" s="60"/>
       <c r="M12" s="60"/>
       <c r="N12" s="80"/>
     </row>
-    <row r="13" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="72"/>
       <c r="B13" s="73">
         <f t="shared" si="0"/>
@@ -2029,392 +2047,414 @@
         <v>37</v>
       </c>
       <c r="E13" s="75" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F13" s="75" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G13" s="75" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H13" s="75" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I13" s="75" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J13" s="82" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K13" s="82" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L13" s="76"/>
       <c r="M13" s="76"/>
       <c r="N13" s="81"/>
     </row>
-    <row r="14" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="38"/>
       <c r="B14" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="61">
-        <v>2</v>
+      <c r="C14" s="61" t="s">
+        <v>131</v>
       </c>
       <c r="D14" s="56" t="s">
-        <v>38</v>
+        <v>139</v>
       </c>
       <c r="E14" s="56" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F14" s="56" t="s">
-        <v>58</v>
+        <v>138</v>
       </c>
       <c r="G14" s="57"/>
       <c r="H14" s="57" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
       <c r="I14" s="57" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="J14" s="77" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K14" s="77" t="s">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="L14" s="58" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M14" s="58" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="N14" s="79"/>
     </row>
-    <row r="15" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="38"/>
-      <c r="B15" s="50">
-        <f t="shared" si="0"/>
+      <c r="B15" s="49">
         <v>6</v>
       </c>
-      <c r="C15" s="62">
-        <v>2</v>
-      </c>
-      <c r="D15" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="59" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" s="59" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="59" t="s">
-        <v>69</v>
-      </c>
-      <c r="H15" s="59" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="J15" s="78" t="s">
-        <v>97</v>
-      </c>
-      <c r="K15" s="78" t="s">
-        <v>105</v>
-      </c>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="80"/>
-    </row>
-    <row r="16" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C15" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="56" t="s">
+        <v>132</v>
+      </c>
+      <c r="E15" s="56" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57" t="s">
+        <v>134</v>
+      </c>
+      <c r="I15" s="57" t="s">
+        <v>83</v>
+      </c>
+      <c r="J15" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="K15" s="77" t="s">
+        <v>135</v>
+      </c>
+      <c r="L15" s="58" t="s">
+        <v>96</v>
+      </c>
+      <c r="M15" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="N15" s="79"/>
+    </row>
+    <row r="16" spans="1:15" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="38"/>
-      <c r="B16" s="49">
+      <c r="B16" s="50">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="61">
-        <v>1</v>
-      </c>
-      <c r="D16" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="56" t="s">
-        <v>51</v>
-      </c>
-      <c r="F16" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="G16" s="57" t="s">
-        <v>70</v>
-      </c>
-      <c r="H16" s="57" t="s">
-        <v>79</v>
-      </c>
-      <c r="I16" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="J16" s="58" t="s">
-        <v>98</v>
-      </c>
-      <c r="K16" s="58" t="s">
-        <v>106</v>
-      </c>
-      <c r="L16" s="77" t="s">
-        <v>97</v>
-      </c>
-      <c r="M16" s="77" t="s">
-        <v>130</v>
-      </c>
-      <c r="N16" s="79"/>
-    </row>
-    <row r="17" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C16" s="62">
+        <v>2</v>
+      </c>
+      <c r="D16" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="59" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="59" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="59" t="s">
+        <v>75</v>
+      </c>
+      <c r="I16" s="59" t="s">
+        <v>86</v>
+      </c>
+      <c r="J16" s="78" t="s">
+        <v>94</v>
+      </c>
+      <c r="K16" s="78" t="s">
+        <v>101</v>
+      </c>
+      <c r="L16" s="60"/>
+      <c r="M16" s="60"/>
+      <c r="N16" s="80"/>
+    </row>
+    <row r="17" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="38"/>
-      <c r="B17" s="50">
+      <c r="B17" s="49">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="62">
+      <c r="C17" s="61">
         <v>1</v>
       </c>
-      <c r="D17" s="59" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="59" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="59" t="s">
-        <v>61</v>
-      </c>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59" t="s">
-        <v>80</v>
-      </c>
-      <c r="I17" s="59" t="s">
-        <v>91</v>
-      </c>
-      <c r="J17" s="60" t="s">
-        <v>99</v>
-      </c>
-      <c r="K17" s="60" t="s">
-        <v>107</v>
-      </c>
-      <c r="L17" s="78" t="s">
-        <v>97</v>
-      </c>
-      <c r="M17" s="78" t="s">
-        <v>131</v>
-      </c>
-      <c r="N17" s="80"/>
-    </row>
-    <row r="18" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="57" t="s">
+        <v>68</v>
+      </c>
+      <c r="H17" s="57" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="57" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="K17" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="L17" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="M17" s="77" t="s">
+        <v>125</v>
+      </c>
+      <c r="N17" s="79"/>
+    </row>
+    <row r="18" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="38"/>
-      <c r="B18" s="49">
+      <c r="B18" s="50">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="61">
+      <c r="C18" s="62">
         <v>1</v>
       </c>
-      <c r="D18" s="56" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="56" t="s">
-        <v>47</v>
-      </c>
-      <c r="F18" s="56" t="s">
-        <v>62</v>
-      </c>
-      <c r="G18" s="57" t="s">
-        <v>71</v>
-      </c>
-      <c r="H18" s="57" t="s">
-        <v>81</v>
-      </c>
-      <c r="I18" s="57" t="s">
-        <v>93</v>
-      </c>
-      <c r="J18" s="77" t="s">
-        <v>97</v>
-      </c>
-      <c r="K18" s="77" t="s">
-        <v>108</v>
-      </c>
-      <c r="L18" s="58"/>
-      <c r="M18" s="58"/>
-      <c r="N18" s="79"/>
-    </row>
-    <row r="19" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" s="59" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="59"/>
+      <c r="H18" s="59" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="J18" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="K18" s="60" t="s">
+        <v>103</v>
+      </c>
+      <c r="L18" s="78" t="s">
+        <v>94</v>
+      </c>
+      <c r="M18" s="78" t="s">
+        <v>126</v>
+      </c>
+      <c r="N18" s="80"/>
+    </row>
+    <row r="19" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="38"/>
-      <c r="B19" s="50">
+      <c r="B19" s="49">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="62" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" s="59" t="s">
-        <v>118</v>
-      </c>
-      <c r="E19" s="59" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="59" t="s">
-        <v>119</v>
-      </c>
-      <c r="G19" s="59"/>
-      <c r="H19" s="59" t="s">
-        <v>121</v>
-      </c>
-      <c r="I19" s="59" t="s">
+      <c r="C19" s="61">
+        <v>1</v>
+      </c>
+      <c r="D19" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="56" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="57" t="s">
+        <v>69</v>
+      </c>
+      <c r="H19" s="57" t="s">
+        <v>78</v>
+      </c>
+      <c r="I19" s="57" t="s">
+        <v>90</v>
+      </c>
+      <c r="J19" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="J19" s="60" t="s">
-        <v>100</v>
-      </c>
-      <c r="K19" s="60" t="s">
-        <v>122</v>
-      </c>
-      <c r="L19" s="78" t="s">
-        <v>97</v>
-      </c>
-      <c r="M19" s="78" t="s">
-        <v>134</v>
-      </c>
-      <c r="N19" s="80"/>
-    </row>
-    <row r="20" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K19" s="77" t="s">
+        <v>104</v>
+      </c>
+      <c r="L19" s="58"/>
+      <c r="M19" s="58"/>
+      <c r="N19" s="79"/>
+    </row>
+    <row r="20" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="38"/>
-      <c r="B20" s="49">
+      <c r="B20" s="50">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="61">
-        <v>1</v>
-      </c>
-      <c r="D20" s="56" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="56" t="s">
-        <v>54</v>
-      </c>
-      <c r="F20" s="56" t="s">
-        <v>63</v>
-      </c>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="I20" s="57" t="s">
-        <v>92</v>
-      </c>
-      <c r="J20" s="58" t="s">
-        <v>54</v>
-      </c>
-      <c r="K20" s="58" t="s">
-        <v>63</v>
-      </c>
-      <c r="L20" s="77" t="s">
+      <c r="C20" s="62" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="59" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" s="59" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="59" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" s="59"/>
+      <c r="H20" s="59" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="59" t="s">
+        <v>91</v>
+      </c>
+      <c r="J20" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="M20" s="77" t="s">
-        <v>132</v>
-      </c>
-      <c r="N20" s="79"/>
-    </row>
-    <row r="21" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K20" s="60" t="s">
+        <v>118</v>
+      </c>
+      <c r="L20" s="78" t="s">
+        <v>94</v>
+      </c>
+      <c r="M20" s="78" t="s">
+        <v>129</v>
+      </c>
+      <c r="N20" s="80"/>
+    </row>
+    <row r="21" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="38"/>
-      <c r="B21" s="50">
+      <c r="B21" s="49">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="62">
+      <c r="C21" s="61">
+        <v>1</v>
+      </c>
+      <c r="D21" s="56" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57" t="s">
+        <v>79</v>
+      </c>
+      <c r="I21" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="J21" s="58" t="s">
+        <v>53</v>
+      </c>
+      <c r="K21" s="58" t="s">
+        <v>61</v>
+      </c>
+      <c r="L21" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="M21" s="77" t="s">
+        <v>127</v>
+      </c>
+      <c r="N21" s="79"/>
+    </row>
+    <row r="22" spans="1:14" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="38"/>
+      <c r="B22" s="50">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C22" s="62">
         <v>2</v>
       </c>
-      <c r="D21" s="59" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" s="59" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="59" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" s="59"/>
-      <c r="H21" s="59" t="s">
-        <v>83</v>
-      </c>
-      <c r="I21" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="J21" s="60" t="s">
-        <v>101</v>
-      </c>
-      <c r="K21" s="60" t="s">
-        <v>64</v>
-      </c>
-      <c r="L21" s="78" t="s">
-        <v>97</v>
-      </c>
-      <c r="M21" s="78" t="s">
-        <v>133</v>
-      </c>
-      <c r="N21" s="80"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" s="38"/>
-      <c r="B22" s="55" t="s">
+      <c r="D22" s="59" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="G22" s="59"/>
+      <c r="H22" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="I22" s="59" t="s">
+        <v>92</v>
+      </c>
+      <c r="J22" s="60" t="s">
+        <v>98</v>
+      </c>
+      <c r="K22" s="60" t="s">
+        <v>62</v>
+      </c>
+      <c r="L22" s="78" t="s">
+        <v>94</v>
+      </c>
+      <c r="M22" s="78" t="s">
+        <v>128</v>
+      </c>
+      <c r="N22" s="80"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="38"/>
+      <c r="B23" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="68"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="5" t="s">
+      <c r="C23" s="68"/>
+      <c r="D23" s="52"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="54"/>
-      <c r="K22" s="54"/>
-      <c r="L22" s="54"/>
-      <c r="M22" s="54"/>
-      <c r="N22" s="53"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="38"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="14"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="J23" s="54"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="54"/>
+      <c r="M23" s="54"/>
+      <c r="N23" s="53"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="38"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
       <c r="M24" s="7"/>
-      <c r="N24" s="15"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="38"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -2423,53 +2463,69 @@
       <c r="F25" s="8"/>
       <c r="G25" s="10"/>
       <c r="H25" s="7"/>
-      <c r="I25" s="7" t="s">
-        <v>21</v>
-      </c>
+      <c r="I25" s="7"/>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
       <c r="N25" s="15"/>
     </row>
-    <row r="26" spans="1:14" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="38"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="16"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="15"/>
+    </row>
+    <row r="27" spans="1:14" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="38"/>
+      <c r="B27" s="33"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="16"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.46" right="0.36" top="0.57999999999999996" bottom="0.984251969" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="60" orientation="landscape" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="63" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;L&amp;BAltium Limited Confidential&amp;B&amp;C&amp;D&amp;RPage &amp;P</oddFooter>
   </headerFooter>
@@ -2481,21 +2537,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="110.5703125" customWidth="1"/>
+    <col min="2" max="2" width="110.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="69" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
@@ -2503,7 +2559,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
@@ -2511,7 +2567,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>3</v>
       </c>
@@ -2519,15 +2575,15 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="71" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>5</v>
       </c>
@@ -2535,7 +2591,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
         <v>6</v>
       </c>
@@ -2543,7 +2599,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
         <v>7</v>
       </c>
@@ -2551,7 +2607,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
         <v>8</v>
       </c>
@@ -2559,44 +2615,44 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="32" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="71" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="70" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="71" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="70" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>